<commit_message>
Atualizacao de arquivos - 26/05/2026 11:33:20,26
</commit_message>
<xml_diff>
--- a/Range CEP.xlsx
+++ b/Range CEP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/pedroofs_algartech_com/Documents/Área de Trabalho/Dashboards/10 - Manutenção Preventiva/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://algarnet-my.sharepoint.com/personal/pedroofs_algartech_com/Documents/Área de Trabalho/Dashboards/9 - Manutenção Preventiva/mp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{AAF38066-702C-4C08-82F9-46B98B948D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EE1D77C-1BF0-4D70-BD8D-FEE9E3E4055E}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{AAF38066-702C-4C08-82F9-46B98B948D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E8CF480-5A78-4246-9C21-CF5DA1CA2DD7}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-2580" windowWidth="24240" windowHeight="13020" xr2:uid="{FE52EA99-E3A3-490C-8D95-E2A65A7C3898}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{FE52EA99-E3A3-490C-8D95-E2A65A7C3898}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$D$763</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -13629,7 +13629,7 @@
         <v>307</v>
       </c>
       <c r="D633" s="1" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
     </row>
     <row r="634" spans="1:4" x14ac:dyDescent="0.25">
@@ -15453,6 +15453,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D763" xr:uid="{023B153A-CD33-4A26-8B28-546D6B298425}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D763">
     <sortCondition ref="A3:A763"/>
   </sortState>

</xml_diff>